<commit_message>
Entrega final Laboratorio 6
</commit_message>
<xml_diff>
--- a/Docs/TablasDatos-Lab6.xlsx
+++ b/Docs/TablasDatos-Lab6.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Universidad\2025-2\Asistencia\Laboratorios\Lab6\ISIS1225-Laboratorio-6\Docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\OneDrive\Documentos\Universidad\Segundo Semestre\EDA\Laboratorio 6\Laboratorio6-G04\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD33DA02-4501-4B58-9D83-E0FFBD1B4D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706C3B4C-C84B-43E7-A76D-FA8F4980782A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="767" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="767" xr2:uid="{D82936D8-D2C9-4EB2-9CBC-3665F65B95FD}"/>
   </bookViews>
   <sheets>
     <sheet name="Datos Lab6" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -116,19 +116,18 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.14999847407452621"/>
-        <bgColor theme="0" tint="-0.14999847407452621"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -169,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -183,16 +182,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -203,6 +196,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,6 +482,1474 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Consumo de Datos [kB] -</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="es-CO" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Linear Probing</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CO"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Datos Lab6'!$B$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Consumo de Datos [kB]</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Datos Lab6'!$A$3:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Datos Lab6'!$B$3:$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>389519.74</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>379504.16</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>378789.82</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>378396</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-3492-4E45-BC5F-CEAF5F6780A4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="546604367"/>
+        <c:axId val="545437967"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="546604367"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="545437967"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="545437967"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="546604367"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CO"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-CO"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-CO" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Consumo de Datos [kB] - Separate Chaining</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CO"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Datos Lab6'!$B$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Consumo de Datos [kB]</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Datos Lab6'!$A$11:$A$14</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Datos Lab6'!$B$11:$B$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>603773.09</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>593439.18999999994</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>590043.61</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>588451.89</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-7B3F-4A37-A737-AD7B0201F3C4}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="825094111"/>
+        <c:axId val="545306447"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="825094111"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="545306447"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="545306447"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="825094111"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CO"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-CO"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-CO" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Tiempo de Ejecución Real [ms] - Linear Probing</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CO"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Datos Lab6'!$C$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Tiempo de Ejecución Real @LP [ms]</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Datos Lab6'!$A$3:$A$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Datos Lab6'!$C$3:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>3908.29</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3667.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3763.35</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4022.93</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-41E0-4BB3-B8BB-45596A17752B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="657341039"/>
+        <c:axId val="545272847"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="657341039"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="545272847"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="545272847"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="657341039"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CO"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-CO"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="es-CO" sz="1400" b="0" i="0" u="none" strike="noStrike" baseline="0"/>
+              <a:t>Tiempo de Ejecución Real [ms] - Separate Chaining</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CO"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Datos Lab6'!$C$10</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Tiempo de Ejecución Real @SC [ms]</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Datos Lab6'!$A$11:$A$14</c:f>
+              <c:numCache>
+                <c:formatCode>0.00</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>8</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Datos Lab6'!$C$11:$C$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>4257.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4568.7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4584.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4629.3500000000004</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-ACEE-4961-8937-72207C1A0DD0}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="713064671"/>
+        <c:axId val="545393807"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="713064671"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="545393807"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="545393807"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="es-CO"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="713064671"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="es-CO"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="es-CO"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="es-ES"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
               <a:rPr lang="es-419" sz="1800" b="1" i="0" baseline="0">
                 <a:effectLst/>
               </a:rPr>
@@ -624,8 +2088,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$B$3:$B$6</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>389519.74</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>379504.16</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>378789.82</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>378396</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -633,8 +2109,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$C$3:$C$6</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>3908.29</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>3667.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3763.35</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4022.93</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -731,8 +2219,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$B$11:$B$14</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>603773.09</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>593439.18999999994</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>590043.61</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>588451.89</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -740,8 +2240,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$C$11:$C$14</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>4257.2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>4568.7</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4584.8</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>4629.3500000000004</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -839,7 +2351,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -964,7 +2476,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1076,7 +2588,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="es-ES"/>
@@ -1297,8 +2809,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$B$3:$B$6</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>389519.74</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>379504.16</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>378789.82</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>378396</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1443,8 +2967,20 @@
             <c:numRef>
               <c:f>'Datos Lab6'!$B$11:$B$14</c:f>
               <c:numCache>
-                <c:formatCode>0.00</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>603773.09</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>593439.18999999994</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>590043.61</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>588451.89</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -1645,7 +3181,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1751,6 +3287,166 @@
 </file>
 
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
   <a:schemeClr val="accent6"/>
   <a:schemeClr val="accent5"/>
@@ -1787,7 +3483,7 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="13">
   <a:schemeClr val="accent6"/>
   <a:schemeClr val="accent5"/>
@@ -1825,7 +3521,7 @@
 </file>
 
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
@@ -1852,8 +3548,8 @@
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
           <a:schemeClr val="tx1">
-            <a:lumMod val="25000"/>
-            <a:lumOff val="75000"/>
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -1954,7 +3650,7 @@
       <a:schemeClr val="tx1"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="19050" cap="rnd">
+      <a:ln w="28575" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
@@ -1986,6 +3682,2018 @@
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="332">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
@@ -2340,7 +6048,7 @@
 </cs:chartStyle>
 </file>
 
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="242">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2836,6 +6544,155 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>600075</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Gráfico 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB754316-10EA-69A3-1F32-3D9F2A40ED9F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>590550</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="3" name="Gráfico 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6BEB3F08-1274-49AD-AD42-5FC00D5C164A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>523874</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Gráfico 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D3C7F8A0-E277-8B41-EBC8-024190F41091}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>9524</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>4762</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="7" name="Gráfico 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{79BBC067-64E6-A725-35FD-B2AA876B4B17}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
@@ -2868,7 +6725,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
@@ -3223,21 +7080,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5B14742-4EBB-4241-AC8A-0E5F24F7BB7B}">
   <dimension ref="A1:C23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="27.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.140625" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:3" ht="18.75">
+      <c r="A1" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
     </row>
-    <row r="2" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="30">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -3248,103 +7105,134 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="8">
+    <row r="3" spans="1:3">
+      <c r="A3" s="6">
         <v>0.1</v>
       </c>
-      <c r="B3" s="5"/>
-      <c r="C3" s="7"/>
+      <c r="B3" s="10">
+        <v>389519.74</v>
+      </c>
+      <c r="C3" s="10">
+        <v>3908.29</v>
+      </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="9">
+    <row r="4" spans="1:3">
+      <c r="A4" s="7">
         <v>0.5</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="7"/>
+      <c r="B4" s="10">
+        <v>379504.16</v>
+      </c>
+      <c r="C4" s="10">
+        <v>3667.5</v>
+      </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="8">
+    <row r="5" spans="1:3">
+      <c r="A5" s="6">
         <v>0.7</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="7"/>
+      <c r="B5" s="10">
+        <v>378789.82</v>
+      </c>
+      <c r="C5" s="10">
+        <v>3763.35</v>
+      </c>
     </row>
-    <row r="6" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="10">
+    <row r="6" spans="1:3" ht="15.75" thickBot="1">
+      <c r="A6" s="8">
         <v>0.9</v>
       </c>
-      <c r="B6" s="2"/>
-      <c r="C6" s="7"/>
+      <c r="B6" s="10">
+        <v>378396</v>
+      </c>
+      <c r="C6" s="10">
+        <v>4022.93</v>
+      </c>
     </row>
-    <row r="9" spans="1:3" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:3" ht="18.75">
+      <c r="A9" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="11"/>
-      <c r="C9" s="11"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
     </row>
-    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="30">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3">
       <c r="A11" s="2">
         <v>2</v>
       </c>
-      <c r="B11" s="2"/>
-      <c r="C11" s="5"/>
+      <c r="B11" s="10">
+        <v>603773.09</v>
+      </c>
+      <c r="C11" s="10">
+        <v>4257.2</v>
+      </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3">
       <c r="A12" s="2">
         <v>4</v>
       </c>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
+      <c r="B12" s="10">
+        <v>593439.18999999994</v>
+      </c>
+      <c r="C12" s="10">
+        <v>4568.7</v>
+      </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3">
       <c r="A13" s="2">
         <v>6</v>
       </c>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
+      <c r="B13" s="10">
+        <v>590043.61</v>
+      </c>
+      <c r="C13" s="10">
+        <v>4584.8</v>
+      </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3">
       <c r="A14" s="2">
         <v>8</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="10">
+        <v>588451.89</v>
+      </c>
+      <c r="C14" s="10">
+        <v>4629.3500000000004</v>
+      </c>
     </row>
-    <row r="23" ht="14.65" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" ht="14.65" customHeight="1"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A9:C9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
   <tableParts count="2">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3597,21 +7485,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="85e30bcc-d76c-4413-8e4d-2dce22fb0743" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="164883f8-7691-4ecf-b54a-664c0d0edefe">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
-    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3636,9 +7523,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F8DF3742-38F2-4B99-B335-CC4F04ED9F45}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97C5E1E0-C817-4769-9D2D-1DC296B681FA}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="85e30bcc-d76c-4413-8e4d-2dce22fb0743"/>
+    <ds:schemaRef ds:uri="164883f8-7691-4ecf-b54a-664c0d0edefe"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>